<commit_message>
Performance-analysis parity + internal significance review
- REVIEW.md: researched internal review (Aug 2026) -- the adapter-selection
  landscape is active (LORAUTER, EdgeLoRA, LoRA-Retriever, LoRAMoE/DLP-LoRA,
  retrieval-based adapter management; routing-free MoE wave); production
  stacks still request-named; lorouter's calibration-competence point is
  unoccupied in the design space; verdict: timely, defensible novelty,
  mechanism-grade evidence; risks and priorities stated plainly
- Workbook upgraded to v2-grade: 9 sheets / 8 charts (was 6/6): Summary
  now carries a reproducibility column per experiment; new CalibrationTrial
  (brick2 vs brick3 full p99/p95 table + chart), ProfileMetric (F9: 73.2%
  vs 96.4% by metric design), AdapterTraining (final losses + variance
  note). README map updated.
</commit_message>
<xml_diff>
--- a/experiments/lorouter_results.xlsx
+++ b/experiments/lorouter_results.xlsx
@@ -11,8 +11,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StandinBenchmark" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RealLoRA" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UnseenTask" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EightAdapter" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalibrationTrial" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProfileMetric" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdapterTraining" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EightAdapter" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,9 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -74,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -82,6 +86,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,6 +503,199 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>p95 thresholds: brick 2 vs brick 3</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>brick 2</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="F87171"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'CalibrationTrial'!$A$5:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'CalibrationTrial'!$B$5:$B$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>brick 3</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2DD4BF"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'CalibrationTrial'!$A$5:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'CalibrationTrial'!$C$5:$C$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Routing accuracy by profile metric</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>accuracy</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="FFB454"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'ProfileMetric'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'ProfileMetric'!$B$5:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Routing accuracy: 4-adapter vs 8-adapter pool</a:t>
             </a:r>
           </a:p>
@@ -569,7 +767,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
@@ -658,7 +856,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
@@ -852,6 +1050,60 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>7</col>
       <colOff>0</colOff>
       <row>3</row>
@@ -875,7 +1127,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1213,12 +1465,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1251,6 +1504,11 @@
           <t>Source script</t>
         </is>
       </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Reproducibility</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1268,6 +1526,11 @@
           <t>experiments/benchmark.py</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pattern exact; digits stable across 5 seeds</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1285,6 +1548,11 @@
           <t>experiments/benchmark.py</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1302,6 +1570,11 @@
           <t>experiments/real_lora_integration.py</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>routing pattern exact across runs; loss digits vary run-to-run (GPU nondeterminism)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1319,6 +1592,11 @@
           <t>experiments/unseen_task_generalization.py</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>distribution exact; quality numbers pattern-level</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1336,6 +1614,11 @@
           <t>experiments/lora_exemplar_routing.py</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>pattern exact; loss digits vary</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1353,6 +1636,11 @@
           <t>experiments/eight_adapter_space.py</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>pattern exact</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1368,6 +1656,33 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>scripts/build_moat_corpus.py + scripts/moat_calibration_trial.py</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>exact (seeded, deterministic)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Profile-metric design (F9)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>question-only loss profiles -&gt; 73.2% routing (code 0%); answer-conditional -&gt; 96.4%</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>experiments/real_lora_integration.py</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>pattern exact</t>
         </is>
       </c>
     </row>
@@ -1864,20 +2179,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Eight-adapter pool (2/domain)</t>
+          <t>Gate calibration -- brick 2 vs brick 3</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Disjoint training data per variant, different answer wording. Domain-level accuracy is the meaningful metric (both variants correct).</t>
+          <t>scripts/moat_calibration_trial.py, gate for education, TF-IDF+SVD+MLP. The s8 property: boundary-inclusive calibration raises the threshold and kills false-capture.</t>
         </is>
       </c>
     </row>
@@ -1889,96 +2204,226 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>brick 2 (n_cal 42)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>brick 3 (n_cal ~110)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>s8 canonical</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>domain-level routing accuracy</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>0.964</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>54/56; identical to 4-adapter pool</t>
-        </is>
+          <t>p99 clean-only threshold</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.3048</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0.8439</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.0031</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>profile min pairwise cosine</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>near-duplicate adapters -&gt; near-identical profiles</t>
-        </is>
+          <t>p99 clean+boundary threshold</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0.9393</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.9943</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>profile mean pairwise cosine</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>separation bounded by adapter diversity</t>
-        </is>
+          <t>p99 false-capture clean-only</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.0476</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>swap isolation (code_A swapped)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+          <t>p99 false-capture clean+boundary</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0/56 routing flips on other domains</t>
-        </is>
+      <c r="C8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>variant split (routed, info only)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>code 0A/13B, edu 16A/0B, fin 0A/14B, law 13A/0B</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>router consistently prefers one variant per domain</t>
-        </is>
+          <t>p99 recall clean-only</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>source: experiments/eight_adapter_space.py</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>p99 recall clean+boundary</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>p95 clean-only threshold</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.1361</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.1283</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>p95 clean+boundary threshold</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.9353</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.6029</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>p95 false-capture clean-only</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.0476</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>0.029</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>p95 false-capture clean+boundary</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>p95 recall clean-only</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>p95 recall clean+boundary</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>addition flips (joint retrain, part 1)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>see s6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>education-boundary escalation (p99)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1 of 7</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1 of 17</t>
         </is>
       </c>
     </row>
@@ -1994,6 +2439,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Profile metric design (finding F9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>experiments/real_lora_integration.py, same adapters, two profile definitions. Profiles must measure ANSWER behavior, not question text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>profile metric</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>routing accuracy</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>code domain</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>question-only NLL (early design)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>near-uniform profiles after normalization; code collapsed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>answer-conditional NLL (current)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>signal restored; matches stand-in benchmark</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Adapter training outcomes (final losses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SmolLM2-135M-Instruct, rank 8, 10 epochs, 62 QA pairs per domain (4-adapter runs; 31 per variant in the 8-adapter run). GPU nondeterminism: digits vary run-to-run, patterns stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>adapter</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>final train loss (4-adapter run)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>final train loss (8-adapter run)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>code-prior base model favors this domain for all adapters</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.473</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>steepest descent; overfits its own QA style</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1.555</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>law</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.389</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>code_A / code_B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1.477 / (B)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>8-adapter variants trained on 31 QA pairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>law_A / law_B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>(A) / 1.582</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Eight-adapter pool (2/domain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Disjoint training data per variant, different answer wording. Domain-level accuracy is the meaningful metric (both variants correct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>domain-level routing accuracy</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>54/56; identical to 4-adapter pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>profile min pairwise cosine</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>near-duplicate adapters -&gt; near-identical profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>profile mean pairwise cosine</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>separation bounded by adapter diversity</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>swap isolation (code_A swapped)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0/56 routing flips on other domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>variant split (routed, info only)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>code 0A/13B, edu 16A/0B, fin 0A/14B, law 13A/0B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>router consistently prefers one variant per domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>source: experiments/eight_adapter_space.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Gap closure: multiseed, model-scale, semantic, latency, generation quality
Five experiments closing every gap the review named (F26-F31):
- real_lora_multiseed.py: 96.4% across seeds 42/7/2026 (F26)
- real_lora_360m.py: 96.4% on SmolLM2-360M, identical to 135M (F27)
- semantic_embeddings.py: profile 98.2% beats centroid 96.4% (ranking
  flip vs lexical, F28); F12 artifact gone - education exemplars route
  to finance (F29)
- latency_spike.py: profiling 1.14ms, cosine 17us->380us (4->10k),
  e2e 2.78ms at 10k (F30)
- generation_quality.py: aligned adapter best output (0.5932 vs 0.5887,
  +0.45pp; F31) - margin small at 135M, stated as such

Workbook now 14 sheets / 11 charts; FINDINGS 31 findings; REVIEW gains
gap-closure status section; README status + limits updated.
</commit_message>
<xml_diff>
--- a/experiments/lorouter_results.xlsx
+++ b/experiments/lorouter_results.xlsx
@@ -14,8 +14,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalibrationTrial" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProfileMetric" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdapterTraining" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EightAdapter" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SemanticBenchmark" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UnseenSemantic" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelScale" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GenerationQuality" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EightAdapter" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,10 +29,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -78,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,6 +93,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -208,6 +215,204 @@
           <val>
             <numRef>
               <f>'StandinBenchmark'!$G$5:$G$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Corpus growth across bricks</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Corpus'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Corpus'!$A$5:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Corpus'!$B$5:$B$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Calibration thresholds: brick 2 vs brick 3 (p95)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>clean-only</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="F87171"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Corpus'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Corpus'!$G$5:$G$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>clean+boundary</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2DD4BF"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Corpus'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Corpus'!$H$5:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -696,6 +901,288 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Semantic vs TF-IDF features: profile routing</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>semantic</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2DD4BF"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'SemanticBenchmark'!$A$5:$A$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SemanticBenchmark'!$B$5:$B$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>TF-IDF+SVD</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="F87171"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'SemanticBenchmark'!$A$5:$A$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SemanticBenchmark'!$C$5:$C$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Selection latency vs pool size</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Latency'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Latency'!$A$5:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Latency'!$B$5:$B$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Generation similarity to reference by adapter</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>similarity</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="FFB454"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'GenerationQuality'!$A$5:$A$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'GenerationQuality'!$B$5:$B$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Routing accuracy: 4-adapter vs 8-adapter pool</a:t>
             </a:r>
           </a:p>
@@ -767,204 +1254,6 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="12"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Corpus growth across bricks</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Corpus'!B4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Corpus'!$A$5:$A$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Corpus'!$B$5:$B$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Calibration thresholds: brick 2 vs brick 3 (p95)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <v>clean-only</v>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="F87171"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Corpus'!$A$5:$A$6</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Corpus'!$G$5:$G$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>clean+boundary</v>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2DD4BF"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Corpus'!$A$5:$A$6</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Corpus'!$H$5:$H$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="80"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -984,6 +1273,55 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1104,7 +1442,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -1131,7 +1469,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -1151,23 +1489,55 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
+        <cNvPr id="1" name="Chart 1"/>
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1691,6 +2061,605 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model-size + seed invariance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>real_lora_multiseed.py (seeds 42/7/2026) + real_lora_360m.py. Routing accuracy is stable across seeds and model sizes (F26, F27).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>seeds</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>routing acc</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>diagonal dominance</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SmolLM2-135M</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>42, 7, 2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>96.4 / 96.4 / 96.4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1/4 each</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SmolLM2-360M</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>96.4%</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Selection-policy latency spike</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>experiments/latency_spike.py, warm mean of 1000 queries. Policy is sub-ms at any realistic pool size (F30).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>pool size N</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>cosine selection (us)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>query profiling (ms)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>end-to-end (ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.157</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.167</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>100</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.165</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.205</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>379.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.775</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Aligned-adapter generation quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>experiments/generation_quality.py: education held out, generations scored by bge-small similarity to reference (F31).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>adapter</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>mean similarity</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>education (aligned)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.5931999999999999</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>routed choice; best output; only domain-plausible continuation in samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>code (best incumbent)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.5887</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>law</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.5839</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>random expectation 0.5862</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.5792</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Eight-adapter pool (2/domain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Disjoint training data per variant, different answer wording. Domain-level accuracy is the meaningful metric (both variants correct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>domain-level routing accuracy</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>54/56; identical to 4-adapter pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>profile min pairwise cosine</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>near-duplicate adapters -&gt; near-identical profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>profile mean pairwise cosine</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>separation bounded by adapter diversity</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>swap isolation (code_A swapped)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0/56 routing flips on other domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>variant split (routed, info only)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>code 0A/13B, edu 16A/0B, fin 0A/14B, law 13A/0B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>router consistently prefers one variant per domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>source: experiments/eight_adapter_space.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Moat corpus growth + calibration stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bricks built by scripts/build_moat_corpus.py (seeded, deterministic). Thresholds from scripts/moat_calibration_trial.py (gate: education).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>brick</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>total examples</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>boundaries</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>calibration split</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>p99 clean-only thr</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>p99 false-capture</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>p95 clean-only thr</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>p95 clean+boundary thr</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>brick 1</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>181</v>
+      </c>
+      <c r="C5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>70/15/15 (n~32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>brick 2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>408</v>
+      </c>
+      <c r="C6" t="n">
+        <v>48</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>70/15/15 (n=80)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.3048</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0476</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.1361</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.9353</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>brick 3</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>664</v>
+      </c>
+      <c r="C7" t="n">
+        <v>64</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>60/25/15 (n=180)</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.8439</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.1283</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.6029</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>brick 2 -&gt; 3: small-n p99 degeneracy resolved (threshold 0.30-&gt;0.84, false-capture 4.76%-&gt;0.00%); boundary value now visible at p95.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2658,35 +3627,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Eight-adapter pool (2/domain)</t>
+          <t>Semantic embeddings arm (bge-small-en-v1.5)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Disjoint training data per variant, different answer wording. Domain-level accuracy is the meaningful metric (both variants correct).</t>
+          <t>experiments/semantic_embeddings.py, brick 2, 5 seeds (same corpus as the TF-IDF benchmark -- like-for-like). Semantic features improve profile routing to 98.2% and flip the centroid ranking (F28).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>strategy</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>semantic acc</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF+SVD acc</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2695,84 +3669,68 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>domain-level routing accuracy</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>0.964</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>54/56; identical to 4-adapter pool</t>
+          <t>profile (lorouter)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.9821</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>now BEATS centroid; ties learned</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>profile min pairwise cosine</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>near-duplicate adapters -&gt; near-identical profiles</t>
+          <t>centroid (embedding)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.9786</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ranking flipped vs lexical features</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>profile mean pairwise cosine</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>separation bounded by adapter diversity</t>
-        </is>
-      </c>
+          <t>learned router</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.9821</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>swap isolation (code_A swapped)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0/56 routing flips on other domains</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>variant split (routed, info only)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>code 0A/13B, edu 16A/0B, fin 0A/14B, law 13A/0B</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>router consistently prefers one variant per domain</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>source: experiments/eight_adapter_space.py</t>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.1929</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.1929</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>floor</t>
         </is>
       </c>
     </row>
@@ -2788,152 +3746,75 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Moat corpus growth + calibration stability</t>
+          <t>Unseen-task exemplar routing: F12 retest</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bricks built by scripts/build_moat_corpus.py (seeded, deterministic). Thresholds from scripts/moat_calibration_trial.py (gate: education).</t>
+          <t>experiments/semantic_embeddings.py. The lexical artifact (all-&gt;code) disappears with semantic task embeddings (F29).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>brick</t>
+          <t>features</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>total examples</t>
+          <t>task-level (10 exemplars)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>boundaries</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>calibration split</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>p99 clean-only thr</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>p99 false-capture</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>p95 clean-only thr</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>p95 clean+boundary thr</t>
+          <t>per-query distribution</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>brick 1</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>181</v>
-      </c>
-      <c r="C5" t="n">
-        <v>17</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>70/15/15 (n~32)</t>
+          <t>TF-IDF+SVD (old)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>code (artifact)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>finance 10, code 2, law 2</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>brick 2</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>408</v>
-      </c>
-      <c r="C6" t="n">
-        <v>48</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>70/15/15 (n=80)</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0.3048</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.0476</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.1361</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.9353</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>brick 3</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>664</v>
-      </c>
-      <c r="C7" t="n">
-        <v>64</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>60/25/15 (n=180)</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0.8439</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.1283</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.6029</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>brick 2 -&gt; 3: small-n p99 degeneracy resolved (threshold 0.30-&gt;0.84, false-capture 4.76%-&gt;0.00%); boundary value now visible at p95.</t>
+          <t>bge-small-en-v1.5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>finance (sensible)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>finance 6, code 3, law 5</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adapter-pool scaling to 1024: the settling test (F32-F36)
adapter_pool_scaling.py: variant profiles = real-LoRA base profiles +
Gaussian noise sigma, N=8..1024, 5 seeds, 92 brick-3 queries.
Findings: (32) zero-noise accuracy FLAT at 96.74% 8->1024 -- pool size
per se is not the failure driver; (33) U-shaped curve under noise
(variant multiplicity helps, extreme-N max-of-N decays); (34) the key
law -- Bonferroni-style compounding does NOT transfer to adapter pools,
measured false capture far below naive independence (correlated
variants); (35) swap isolation 0.00% at N=128/512; (36) separation min
collapses with noise, mean stable. Workbook +15 sheets/12 charts with
PoolScaling line chart; REVIEW + README updated.
</commit_message>
<xml_diff>
--- a/experiments/lorouter_results.xlsx
+++ b/experiments/lorouter_results.xlsx
@@ -19,8 +19,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelScale" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GenerationQuality" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EightAdapter" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PoolScaling" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EightAdapter" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -256,6 +257,90 @@
 
 <file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Routing accuracy: 4-adapter vs 8-adapter pool</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>accuracy</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2DD4BF"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'EightAdapter'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'EightAdapter'!$B$5:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
     <title>
@@ -343,7 +428,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
@@ -1172,7 +1257,7 @@
 
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="12"/>
   <chart>
     <title>
       <tx>
@@ -1183,45 +1268,138 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Routing accuracy: 4-adapter vs 8-adapter pool</a:t>
+              <a:t>Routing accuracy vs pool size (by sigma)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
+      <lineChart>
+        <grouping val="standard"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>accuracy</v>
+            <v>sigma=0.0</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2DD4BF"/>
-            </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
-              <f>'EightAdapter'!$A$5:$A$6</f>
+              <f>'PoolScaling'!$A$5:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EightAdapter'!$B$5:$B$6</f>
+              <f>'PoolScaling'!$C$5:$C$9</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="80"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>sigma=0.05</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'PoolScaling'!$A$5:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PoolScaling'!$C$10:$C$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>sigma=0.1</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'PoolScaling'!$A$5:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PoolScaling'!$C$15:$C$19</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>sigma=0.2</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'PoolScaling'!$A$5:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PoolScaling'!$C$20:$C$24</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
-      </barChart>
+      </lineChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -1282,6 +1460,33 @@
 </file>
 
 <file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1528,7 +1733,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3240000"/>
+    <ext cx="7920000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -2380,122 +2585,453 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Eight-adapter pool (2/domain)</t>
+          <t>Adapter-pool scaling (F32-F36)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Disjoint training data per variant, different answer wording. Domain-level accuracy is the meaningful metric (both variants correct).</t>
+          <t>experiments/adapter_pool_scaling.py: variant profiles = real-LoRA base profiles + Gaussian noise sigma, 5 seeds, 92 brick-3 queries. U-shaped accuracy: sigma=0 flat at 96.7%; noise -&gt; mid-N helps, extreme-N decays.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>sigma</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>false_capture</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>sep_min</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>sep_mean</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>domain-level routing accuracy</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>0.964</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>54/56; identical to 4-adapter pool</t>
-        </is>
+      <c r="A5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.9674</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.996</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>profile min pairwise cosine</t>
-        </is>
+      <c r="A6" t="n">
+        <v>32</v>
       </c>
       <c r="B6" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>near-duplicate adapters -&gt; near-identical profiles</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.9674</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.997</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>profile mean pairwise cosine</t>
-        </is>
+      <c r="A7" t="n">
+        <v>128</v>
       </c>
       <c r="B7" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>separation bounded by adapter diversity</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.9674</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.997</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>swap isolation (code_A swapped)</t>
-        </is>
+      <c r="A8" t="n">
+        <v>512</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0/56 routing flips on other domains</t>
-        </is>
+      <c r="C8" s="6" t="n">
+        <v>0.9674</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.997</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>variant split (routed, info only)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>code 0A/13B, edu 16A/0B, fin 0A/14B, law 13A/0B</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>router consistently prefers one variant per domain</t>
-        </is>
+      <c r="A9" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.9674</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.997</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>source: experiments/eight_adapter_space.py</t>
-        </is>
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.3957</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.6042999999999999</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.964</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>32</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.5978</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.4022</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.968</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>128</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>0.7739</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0.2261</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.968</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>512</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>0.7304</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0.2696</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.968</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0.6565</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.3435</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.715</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.968</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.883</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>32</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>0.4391</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>0.5609</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.431</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.886</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>128</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.887</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>512</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>0.4391</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>0.5609</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.887</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>0.4761</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>0.5239</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-0.065</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.885</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0.3717</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>0.6283</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.641</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>32</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>0.3804</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>0.6196</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-0.479</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.639</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>128</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>0.3891</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0.6109</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-0.827</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.642</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>512</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-0.982</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.635</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>0.3043</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>0.6957</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-0.997</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.63</v>
       </c>
     </row>
   </sheetData>
@@ -2505,6 +3041,136 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Eight-adapter pool (2/domain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Disjoint training data per variant, different answer wording. Domain-level accuracy is the meaningful metric (both variants correct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>domain-level routing accuracy</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>54/56; identical to 4-adapter pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>profile min pairwise cosine</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>near-duplicate adapters -&gt; near-identical profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>profile mean pairwise cosine</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>separation bounded by adapter diversity</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>swap isolation (code_A swapped)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0/56 routing flips on other domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>variant split (routed, info only)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>code 0A/13B, edu 16A/0B, fin 0A/14B, law 13A/0B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>router consistently prefers one variant per domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>source: experiments/eight_adapter_space.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Docs consistency pass: kill stale references on lorouter
- brick correction: real-LoRA experiments ran on the loader's default
  corpus (brick 2), not brick 3 -- fixed README status, FINDINGS F31 note,
  LOROUTER 3.2, real_lora_integration.py + eight_adapter_space.py
  docstrings; moat_calibration_trial.py docstring now says brick 3 (its
  code was already pointed there)
- FINDINGS header dates 2026-08-05/06
- LOROUTER 3.3/3.4: unseen-task quality now verified at aligned level
  (F13/F31); pool scaling added; limits section updated (semantic arm,
  latency, aligned-level quality)
- possibility.md: evidence table +7 rows (multi-seed/360M, semantic,
  latency, gen quality, pool scaling); roadmap marked DONE/open
- REVIEW.md: priority list statused; workbook Summary date + unseen row
- README layout: all 12 experiments + results/ listed; sheet count 15
</commit_message>
<xml_diff>
--- a/experiments/lorouter_results.xlsx
+++ b/experiments/lorouter_results.xlsx
@@ -2059,7 +2059,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Canonical run 2026-08-05, lorouter branch. Scripts are the source of truth.</t>
+          <t>Canonical runs 2026-08-05/06, lorouter branch. Scripts are the source of truth.</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2159,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>routing stable: education-&gt;finance 10/14 (real + stand-in arms agree); oracle agreement 42.9%; loss gap == random (quality OPEN)</t>
+          <t>routing stable: education-&gt;finance 10/14 (real + stand-in arms agree); quality verified at the aligned-adapter level (F13/F31); without aligned adapter the loss gap == random</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>

<commit_message>
v3 corpus (user-built, 3,010 ex / 6 domains / 220 boundaries): verified + documented
User extended the corpus 4.5x (medicine + psychology added). Verified:
- integrity: 3,010 unique ids/texts, zero leakage, schema-compliant
- boundary hardness at scale: 94.0% clean vs 0.0% boundary (F38)
- calibration on v3 (p99): 0.0448 -> 0.7638, fc 1.79% -> 0.00%, recall
  97.3% -> 93.3% (F39); p95 effect real but weaker (six-domain space
  harder); escalation 6/34 (F40); addition flips 7 (F41)
FINDINGS F37-F41 (section I); docs stats updated everywhere (README,
LOROUTER, possibility, TECHNICAL appendix incl. generator provenance
note); workbook Corpus/CalibrationTrial/Summary sheets updated; H-section
provenance note (pool scaling ran pre-v3). real_lora_six_domain.py added
(running); ANSWERS extended with medicine/psychology templates.
</commit_message>
<xml_diff>
--- a/experiments/lorouter_results.xlsx
+++ b/experiments/lorouter_results.xlsx
@@ -2220,22 +2220,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Corpus brick 3 (664 ex, 25% calib split)</t>
+          <t>Corpus brick 3 v3 (user-built)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>p99 clean-only threshold 0.30-&gt;0.84, false-capture 4.76%-&gt;0.00% vs brick 2 (degeneracy resolved)</t>
+          <t>3,010 ex / 6 domains / 220 boundaries; boundary hardness 94.0% clean vs 0.0% boundary; p99 clean-only threshold 0.0448 -&gt; 0.7638, false-capture 1.79% -&gt; 0.00%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>scripts/build_moat_corpus.py + scripts/moat_calibration_trial.py</t>
+          <t>corpus/moat_brick3.jsonl + scripts/moat_calibration_trial.py</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>exact (seeded, deterministic)</t>
+          <t>exact (seeded/deterministic parts); v3 file fixed</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3286,7 +3286,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>brick 3</t>
+          <t>brick 3 (pre-v3)</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3313,10 +3313,47 @@
         <v>0.6029</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>brick 3 v3 (user-built)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3010</v>
+      </c>
+      <c r="C8" t="n">
+        <v>220</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1673/807/530 (n~135/domain)</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0179</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0594</v>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>brick 2 -&gt; 3: small-n p99 degeneracy resolved (threshold 0.30-&gt;0.84, false-capture 4.76%-&gt;0.00%); boundary value now visible at p95.</t>
+          <t>brick 2 -&gt; pre-v3: small-n p99 degeneracy resolved. v3 (user-built, 6 domains + medicine/psychology): the six-domain space is harder -- p99 false-capture 1.79% -&gt; 0.00% with boundaries; p95 effect real but weaker (4.02% -&gt; 1.34%). Addition flips at v3: 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>v3 integrity: 3,010 unique ids/texts, zero calib/test leakage into train; boundary hardness 94.0% clean vs 0.0% boundary (F37-F41).</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3881,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>brick 3 (n_cal ~110)</t>
+          <t>v3 brick 3 (n_cal ~135/domain)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3863,7 +3900,7 @@
         <v>0.3048</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>0.8439</v>
+        <v>0.0448</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>0.0031</v>
@@ -3879,7 +3916,7 @@
         <v>0.992</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.9393</v>
+        <v>0.7638</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>0.9943</v>
@@ -3895,7 +3932,7 @@
         <v>0.0476</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>0</v>
+        <v>0.0179</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>0.016</v>
@@ -3927,7 +3964,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.957</v>
+        <v>0.973</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>1</v>
@@ -3943,7 +3980,7 @@
         <v>0.714</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>0.826</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>0.92</v>
@@ -3959,7 +3996,7 @@
         <v>0.1361</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>0.1283</v>
+        <v>0.0032</v>
       </c>
     </row>
     <row r="12">
@@ -3972,7 +4009,7 @@
         <v>0.9353</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>0.6029</v>
+        <v>0.0594</v>
       </c>
     </row>
     <row r="13">
@@ -3985,7 +4022,7 @@
         <v>0.0476</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>0.029</v>
+        <v>0.0402</v>
       </c>
     </row>
     <row r="14">
@@ -3998,7 +4035,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>0</v>
+        <v>0.0134</v>
       </c>
     </row>
     <row r="15">
@@ -4011,7 +4048,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1</v>
+        <v>0.987</v>
       </c>
     </row>
     <row r="16">
@@ -4024,7 +4061,7 @@
         <v>0.929</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>1</v>
+        <v>0.973</v>
       </c>
     </row>
     <row r="17">
@@ -4037,7 +4074,7 @@
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -4058,7 +4095,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1 of 17</t>
+          <t>6 of 34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Six-domain real-LoRA scale-up on v3 corpus (F42): 95.7% routing, 6/6 diagonal
Six adapters on the user's v3 corpus (230-300 QA pairs/domain): routing
95.7% (402/420, per-domain 93.3-98.4%, random floor 16.7%) - the 4-domain
96.4% holds within ~1 point. Loss matrix fully diagonal (medicine 0.55 on
own domain vs 2.1+ elsewhere). KEY REVISION: the F7/F8 'base-model priors
bound differentiation' finding was a data-volume bound - at ~5x training
data, every adapter is its own-domain specialist. LOROUTER 3.2, README
status, workbook ModelScale updated.
</commit_message>
<xml_diff>
--- a/experiments/lorouter_results.xlsx
+++ b/experiments/lorouter_results.xlsx
@@ -2272,7 +2272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2352,6 +2352,28 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>2/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SmolLM2-135M, 6 domains (v3 corpus, F42)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>95.7% (402/420)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>6/6</t>
         </is>
       </c>
     </row>

</xml_diff>